<commit_message>
new config of paper searching + paper extraction (rag by chunk + iteration on best terms)
</commit_message>
<xml_diff>
--- a/count_new_paper_by_disease.xlsx
+++ b/count_new_paper_by_disease.xlsx
@@ -22,13 +22,13 @@
     <t>Count papers</t>
   </si>
   <si>
+    <t>Alzheimer Disease</t>
+  </si>
+  <si>
+    <t>Parkinson Disease</t>
+  </si>
+  <si>
     <t>Other ADRD</t>
-  </si>
-  <si>
-    <t>Alzheimer Disease</t>
-  </si>
-  <si>
-    <t>Parkinson Disease</t>
   </si>
   <si>
     <t>Amyotrophic Lateral Sclerosis</t>
@@ -408,7 +408,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>631</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -416,7 +416,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>468</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -424,7 +424,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>83</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -432,7 +432,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>59</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -440,7 +440,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>